<commit_message>
Remove Selling Unit from Add Stock and bulk upload, and auto-generate Barcodes
</commit_message>
<xml_diff>
--- a/sample_bulk_upload_products.xlsx
+++ b/sample_bulk_upload_products.xlsx
@@ -397,341 +397,273 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:G11"/>
   <cols>
-    <col min="1" max="1" width="14.83203125" customWidth="1"/>
-    <col min="2" max="2" width="16.83203125" customWidth="1"/>
-    <col min="3" max="3" width="14.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="14.83203125" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" customWidth="1"/>
+    <col min="1" max="1" width="16.83203125" customWidth="1"/>
+    <col min="2" max="2" width="15.83203125" customWidth="1"/>
+    <col min="3" max="3" width="15.83203125" customWidth="1"/>
+    <col min="4" max="4" width="15.83203125" customWidth="1"/>
+    <col min="5" max="5" width="15.83203125" customWidth="1"/>
+    <col min="6" max="6" width="17.83203125" customWidth="1"/>
     <col min="7" max="7" width="17.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="17.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Barcode</v>
+        <v>Product Name</v>
       </c>
       <c r="B1" t="str">
-        <v>Product Name</v>
+        <v>Category</v>
       </c>
       <c r="C1" t="str">
-        <v>Category</v>
+        <v>Cost</v>
       </c>
       <c r="D1" t="str">
-        <v>Cost</v>
+        <v>Markup</v>
       </c>
       <c r="E1" t="str">
-        <v>Markup</v>
+        <v>Price</v>
       </c>
       <c r="F1" t="str">
-        <v>Price</v>
+        <v>Current Stock</v>
       </c>
       <c r="G1" t="str">
-        <v>Current Stock</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Selling Unit</v>
-      </c>
-      <c r="I1" t="str">
         <v>Reorder Level</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>LEG-00101</v>
+        <v>Portland Cement (50kg Bag)</v>
       </c>
       <c r="B2" t="str">
-        <v>Portland Cement (50kg Bag)</v>
-      </c>
-      <c r="C2" t="str">
         <v>Building Materials</v>
       </c>
-      <c r="D2">
+      <c r="C2">
         <v>85</v>
       </c>
-      <c r="E2" t="str">
+      <c r="D2" t="str">
         <v>29%</v>
       </c>
+      <c r="E2">
+        <v>110</v>
+      </c>
       <c r="F2">
-        <v>110</v>
+        <v>200</v>
       </c>
       <c r="G2">
-        <v>200</v>
-      </c>
-      <c r="H2" t="str">
-        <v>Bag</v>
-      </c>
-      <c r="I2">
         <v>50</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>LEG-00102</v>
+        <v>High Tensile Steel Rod 12mm</v>
       </c>
       <c r="B3" t="str">
-        <v>High Tensile Steel Rod 12mm</v>
-      </c>
-      <c r="C3" t="str">
         <v>Building Materials</v>
       </c>
-      <c r="D3">
+      <c r="C3">
         <v>60</v>
       </c>
-      <c r="E3" t="str">
+      <c r="D3" t="str">
         <v>30%</v>
       </c>
+      <c r="E3">
+        <v>78</v>
+      </c>
       <c r="F3">
-        <v>78</v>
+        <v>150</v>
       </c>
       <c r="G3">
-        <v>150</v>
-      </c>
-      <c r="H3" t="str">
-        <v>Piece</v>
-      </c>
-      <c r="I3">
         <v>30</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>LEG-00103</v>
+        <v>PVC Pressure Pipe 4 Inch (6m)</v>
       </c>
       <c r="B4" t="str">
-        <v>PVC Pressure Pipe 4 Inch (6m)</v>
-      </c>
-      <c r="C4" t="str">
         <v>Plumbing Supplies</v>
       </c>
-      <c r="D4">
+      <c r="C4">
         <v>45</v>
       </c>
-      <c r="E4" t="str">
+      <c r="D4" t="str">
         <v>44%</v>
       </c>
+      <c r="E4">
+        <v>65</v>
+      </c>
       <c r="F4">
-        <v>65</v>
+        <v>80</v>
       </c>
       <c r="G4">
-        <v>80</v>
-      </c>
-      <c r="H4" t="str">
-        <v>Length</v>
-      </c>
-      <c r="I4">
         <v>20</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>LEG-00104</v>
+        <v>Acrylic Emulsion Paint White (20L)</v>
       </c>
       <c r="B5" t="str">
-        <v>Acrylic Emulsion Paint White (20L)</v>
-      </c>
-      <c r="C5" t="str">
         <v>Paints &amp; Finishes</v>
       </c>
-      <c r="D5">
+      <c r="C5">
         <v>280</v>
       </c>
-      <c r="E5" t="str">
+      <c r="D5" t="str">
         <v>28%</v>
       </c>
+      <c r="E5">
+        <v>360</v>
+      </c>
       <c r="F5">
-        <v>360</v>
+        <v>40</v>
       </c>
       <c r="G5">
-        <v>40</v>
-      </c>
-      <c r="H5" t="str">
-        <v>Bucket</v>
-      </c>
-      <c r="I5">
         <v>10</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>LEG-00105</v>
+        <v>Claw Hammer 16oz Fiberglass</v>
       </c>
       <c r="B6" t="str">
-        <v>Claw Hammer 16oz Fiberglass</v>
-      </c>
-      <c r="C6" t="str">
         <v>Tools &amp; Hardware</v>
       </c>
-      <c r="D6">
+      <c r="C6">
         <v>35</v>
       </c>
-      <c r="E6" t="str">
+      <c r="D6" t="str">
         <v>48%</v>
       </c>
+      <c r="E6">
+        <v>52</v>
+      </c>
       <c r="F6">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="G6">
-        <v>60</v>
-      </c>
-      <c r="H6" t="str">
-        <v>Piece</v>
-      </c>
-      <c r="I6">
         <v>15</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>LEG-00106</v>
+        <v>Angle Grinder 115mm 850W</v>
       </c>
       <c r="B7" t="str">
-        <v>Angle Grinder 115mm 850W</v>
-      </c>
-      <c r="C7" t="str">
         <v>Tools &amp; Hardware</v>
       </c>
-      <c r="D7">
+      <c r="C7">
         <v>220</v>
       </c>
-      <c r="E7" t="str">
+      <c r="D7" t="str">
         <v>40%</v>
       </c>
+      <c r="E7">
+        <v>310</v>
+      </c>
       <c r="F7">
-        <v>310</v>
+        <v>25</v>
       </c>
       <c r="G7">
-        <v>25</v>
-      </c>
-      <c r="H7" t="str">
-        <v>Unit</v>
-      </c>
-      <c r="I7">
         <v>5</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>LEG-00107</v>
+        <v>2.5mm Twin &amp; Earth Cable (100m)</v>
       </c>
       <c r="B8" t="str">
-        <v>2.5mm Twin &amp; Earth Cable (100m)</v>
-      </c>
-      <c r="C8" t="str">
         <v>Electrical Supplies</v>
       </c>
-      <c r="D8">
+      <c r="C8">
         <v>320</v>
       </c>
-      <c r="E8" t="str">
+      <c r="D8" t="str">
         <v>34%</v>
       </c>
+      <c r="E8">
+        <v>430</v>
+      </c>
       <c r="F8">
-        <v>430</v>
+        <v>30</v>
       </c>
       <c r="G8">
-        <v>30</v>
-      </c>
-      <c r="H8" t="str">
-        <v>Roll</v>
-      </c>
-      <c r="I8">
         <v>8</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>LEG-00108</v>
+        <v>Drywall Screws 3.5x25mm (Box 1000)</v>
       </c>
       <c r="B9" t="str">
-        <v>Drywall Screws 3.5x25mm (Box 1000)</v>
-      </c>
-      <c r="C9" t="str">
         <v>Fasteners &amp; Fixings</v>
       </c>
-      <c r="D9">
+      <c r="C9">
         <v>28</v>
       </c>
-      <c r="E9" t="str">
+      <c r="D9" t="str">
         <v>50%</v>
       </c>
+      <c r="E9">
+        <v>42</v>
+      </c>
       <c r="F9">
-        <v>42</v>
+        <v>100</v>
       </c>
       <c r="G9">
-        <v>100</v>
-      </c>
-      <c r="H9" t="str">
-        <v>Box</v>
-      </c>
-      <c r="I9">
         <v>25</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v/>
+        <v>Safety Hard Hat (Yellow)</v>
       </c>
       <c r="B10" t="str">
-        <v>Safety Hard Hat (Yellow)</v>
-      </c>
-      <c r="C10" t="str">
         <v>Safety &amp; PPE</v>
       </c>
-      <c r="D10">
+      <c r="C10">
         <v>25</v>
       </c>
-      <c r="E10" t="str">
+      <c r="D10" t="str">
         <v>40%</v>
       </c>
+      <c r="E10">
+        <v>35</v>
+      </c>
       <c r="F10">
-        <v>35</v>
+        <v>50</v>
       </c>
       <c r="G10">
-        <v>50</v>
-      </c>
-      <c r="H10" t="str">
-        <v>Piece</v>
-      </c>
-      <c r="I10">
         <v>12</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v/>
+        <v>Measuring Tape 8m / 26ft Heavy Duty</v>
       </c>
       <c r="B11" t="str">
-        <v>Measuring Tape 8m / 26ft Heavy Duty</v>
-      </c>
-      <c r="C11" t="str">
         <v>Tools &amp; Hardware</v>
       </c>
-      <c r="D11">
+      <c r="C11">
         <v>22</v>
       </c>
-      <c r="E11" t="str">
+      <c r="D11" t="str">
         <v>45%</v>
       </c>
+      <c r="E11">
+        <v>32</v>
+      </c>
       <c r="F11">
-        <v>32</v>
+        <v>75</v>
       </c>
       <c r="G11">
-        <v>75</v>
-      </c>
-      <c r="H11" t="str">
-        <v>Piece</v>
-      </c>
-      <c r="I11">
         <v>15</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Set default reorder level to 1 and add Date to single and bulk stock entry
</commit_message>
<xml_diff>
--- a/sample_bulk_upload_products.xlsx
+++ b/sample_bulk_upload_products.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:H11"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -406,6 +406,7 @@
     <col min="5" max="5" width="15.83203125" customWidth="1"/>
     <col min="6" max="6" width="17.83203125" customWidth="1"/>
     <col min="7" max="7" width="17.83203125" customWidth="1"/>
+    <col min="8" max="8" width="15.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -430,6 +431,9 @@
       <c r="G1" t="str">
         <v>Reorder Level</v>
       </c>
+      <c r="H1" t="str">
+        <v>Date</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -451,7 +455,10 @@
         <v>200</v>
       </c>
       <c r="G2">
-        <v>50</v>
+        <v>1</v>
+      </c>
+      <c r="H2" t="str">
+        <v>2026-09-24</v>
       </c>
     </row>
     <row r="3">
@@ -474,7 +481,10 @@
         <v>150</v>
       </c>
       <c r="G3">
-        <v>30</v>
+        <v>1</v>
+      </c>
+      <c r="H3" t="str">
+        <v>2026-09-24</v>
       </c>
     </row>
     <row r="4">
@@ -497,7 +507,10 @@
         <v>80</v>
       </c>
       <c r="G4">
-        <v>20</v>
+        <v>1</v>
+      </c>
+      <c r="H4" t="str">
+        <v>2026-09-24</v>
       </c>
     </row>
     <row r="5">
@@ -520,7 +533,10 @@
         <v>40</v>
       </c>
       <c r="G5">
-        <v>10</v>
+        <v>1</v>
+      </c>
+      <c r="H5" t="str">
+        <v>2026-09-24</v>
       </c>
     </row>
     <row r="6">
@@ -543,7 +559,10 @@
         <v>60</v>
       </c>
       <c r="G6">
-        <v>15</v>
+        <v>1</v>
+      </c>
+      <c r="H6" t="str">
+        <v>2026-09-24</v>
       </c>
     </row>
     <row r="7">
@@ -566,7 +585,10 @@
         <v>25</v>
       </c>
       <c r="G7">
-        <v>5</v>
+        <v>1</v>
+      </c>
+      <c r="H7" t="str">
+        <v>2026-09-24</v>
       </c>
     </row>
     <row r="8">
@@ -589,7 +611,10 @@
         <v>30</v>
       </c>
       <c r="G8">
-        <v>8</v>
+        <v>1</v>
+      </c>
+      <c r="H8" t="str">
+        <v>2026-09-24</v>
       </c>
     </row>
     <row r="9">
@@ -612,7 +637,10 @@
         <v>100</v>
       </c>
       <c r="G9">
-        <v>25</v>
+        <v>1</v>
+      </c>
+      <c r="H9" t="str">
+        <v>2026-09-24</v>
       </c>
     </row>
     <row r="10">
@@ -635,7 +663,10 @@
         <v>50</v>
       </c>
       <c r="G10">
-        <v>12</v>
+        <v>1</v>
+      </c>
+      <c r="H10" t="str">
+        <v>2026-09-24</v>
       </c>
     </row>
     <row r="11">
@@ -658,12 +689,15 @@
         <v>75</v>
       </c>
       <c r="G11">
-        <v>15</v>
+        <v>1</v>
+      </c>
+      <c r="H11" t="str">
+        <v>2026-09-24</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>